<commit_message>
feat: designing the generated excel and pdf file
</commit_message>
<xml_diff>
--- a/tithes-report.xlsx
+++ b/tithes-report.xlsx
@@ -4,14 +4,17 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Sheet 1" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Tithes" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
+  <si>
+    <t>JOSCM Tithes Report</t>
+  </si>
   <si>
     <t>Entry Date</t>
   </si>
@@ -28,6 +31,9 @@
     <t>Status</t>
   </si>
   <si>
+    <t>Reviewed By</t>
+  </si>
+  <si>
     <t>Kids Ministry</t>
   </si>
   <si>
@@ -37,6 +43,9 @@
     <t>pending</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>Sunday Service</t>
   </si>
   <si>
@@ -44,13 +53,16 @@
   </si>
   <si>
     <t>Adrian</t>
+  </si>
+  <si>
+    <t>Total Balance:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -58,16 +70,40 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFBBF24"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF34D399"/>
+    </font>
+    <font>
+      <b/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4F8EF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -75,13 +111,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -421,101 +485,137 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="5" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="E2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
         <v>45998</v>
       </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2">
+      <c r="B3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="5">
         <v>8000</v>
       </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
+      <c r="D3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
         <v>45998</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="5">
+        <v>9000</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C3">
+      <c r="E4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>46118</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="5">
         <v>9000</v>
       </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="D5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>9</v>
       </c>
+      <c r="F5" s="5" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>46118</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>46119</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="5">
+        <v>9100</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C4">
-        <v>9000</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s">
-        <v>7</v>
+      <c r="E6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>46119</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5">
-        <v>9100</v>
-      </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" t="s">
-        <v>9</v>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="8">
+        <f>SUM(C3:C6)</f>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>